<commit_message>
feat(workbook): generate SECUI grouped CLI rules
</commit_message>
<xml_diff>
--- a/request-folder/_빈양식/신청서_빈양식.xlsx
+++ b/request-folder/_빈양식/신청서_빈양식.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:M1"/>
+  <dimension ref="B1:N1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -451,55 +451,60 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>대상방화벽</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>출발지IP</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>출발지</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>목적지IP</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>목적지</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>프로토콜</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>포트</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>방향</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>용도</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>시작일</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>종료일</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>비고</t>
         </is>

</xml_diff>